<commit_message>
Auto backup: 2026-08-15 05:19:19
</commit_message>
<xml_diff>
--- a/Tính doanh thu.xlsx
+++ b/Tính doanh thu.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\BuonBanXe\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E4B21597-FE45-469E-AB56-4B5917AE7DCA}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EF76FDC-77AA-419C-A9DB-D0C8CD00FB6F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="10605" xr2:uid="{C3D4EEB7-466F-4B4A-84A8-966289F7C3D7}"/>
   </bookViews>
@@ -415,11 +415,11 @@
     </row>
     <row r="2" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2">
-        <v>6300000</v>
+        <v>7700000</v>
       </c>
       <c r="B2" s="2">
         <f>ROUNDUP(A2 / 0.94, -4)</f>
-        <v>6710000</v>
+        <v>8200000</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2">

</xml_diff>